<commit_message>
Deployed a85998e5f to fix-aesthetics with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/fix-aesthetics/issues_list.xlsx
+++ b/fix-aesthetics/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,7 +460,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -475,7 +475,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -490,7 +490,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -505,7 +505,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -520,361 +520,976 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='2.0' | DataCite='1.0'</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1sqnqvcxxcuqjfqasluneu6r311tfiogw/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work 'https://drive.google.com/file/d/1blzfowqmictyuet4mnip2d2nnmd2pxjg/view?usp=sharing' in CKAN not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1269473 returned status_code=500</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Tentative dataset should not have a version</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ee2eec87-7a78-4a7f-87b7-54347a6c3b2f</t>
+          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf returned status_code=timeout</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Contact missing affiliation: Floyd, William</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Contact missing affiliation: Floyd, William</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Contact missing affiliation: VanMaanen, Derek</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Contact missing affiliation: Liggan, Lauran</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>a31d44d5-2ce5-4d03-8d0b-4549023840ff</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Contact missing affiliation: Millard-Martin, Ben</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>44bdc298-1329-400a-bc02-4d35d251865d</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Contact missing affiliation: Whalen, Matthew</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/q31x-qg72' (References) in DataCite not found in CKAN</t>
+          <t>Contact missing affiliation: Korver, Maartje C.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier '10.21966/v57r-g944' (References) in DataCite not found in CKAN</t>
+          <t>Contact missing affiliation: Floyd, William</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>1be9154a-1497-42eb-8821-b0d63000814c</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Contact missing affiliation: Lertzman, Ken</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>d8754c99-a540-4085-8c66-d9447da5f6e9</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Contact missing affiliation: Saunders, Sari</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>5576c279-6d3a-4323-8104-0e1040d9906c</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Contact missing affiliation: Burt, Jenn</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>98bc62c7-d6a4-42bd-9110-c8021380d8a5</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Contact missing affiliation: Closs, Alana</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>98bc62c7-d6a4-42bd-9110-c8021380d8a5</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Institute' in CKAN record not found in DataCite</t>
+          <t>Contact missing affiliation: Manning, Faye</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
+          <t>98bc62c7-d6a4-42bd-9110-c8021380d8a5</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tentative dataset should not have a version</t>
+          <t>Contact missing affiliation: Whalen, Matthew</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>98bc62c7-d6a4-42bd-9110-c8021380d8a5</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Millard-Martin, Ben</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>98bc62c7-d6a4-42bd-9110-c8021380d8a5</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Rechsteiner, Erin</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>a8f61379-14f9-4ccc-bc9b-4408ba8340d7</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Liggan, Lauran</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>c06cb551-351c-456f-8d0c-c8aab9aec162</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Oliver, Allison</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Hall, Kyle</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Millard-Martin, Ben</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: VanMaanen, Derek</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Whalen, Matthew</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1dfdbadf-6314-4411-8d18-752f6dd920e9</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Liggan, Lauran</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Floyd, William</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>4f1e8eac-8390-44d8-93d6-9263fc1dfcf9</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Floyd, William</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Tank, Suzanne</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>55e7c337-02e8-4200-8ea9-88241d978f96</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Lertzman, Ken</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Korver, Maartje C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Floyd, William</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Oliver, Allison</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Tank, Suzanne</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>f51d96b5-1827-4aab-b1ce-575faff1fd03</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Millard-Martin, Ben</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Korver, Maartje C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>49ec67e4-f7be-4658-b2b6-e4b57d9901df</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Tank, Suzanne</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Evans, Wiley</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Albers, Sam</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Hare, Alex</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Barrette, Jessy</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Jackson, Jennifer</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>9e4a38d6-eb29-44a8-b495-c56ce74a227c</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Hales, Burke</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Whalen, Matthew</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: VanMaanen, Derek</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Liggan, Lauran</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Hall, Kyle</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: VanMaanen, Derek</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Liggan, Lauran</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>967f98cb-131a-421e-bcfd-467cff973b30</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Millard-Martin, Ben</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>967f98cb-131a-421e-bcfd-467cff973b30</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Liggan, Lauran</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>967f98cb-131a-421e-bcfd-467cff973b30</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: VanMaanen, Derek</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>6a6908af-8856-431e-8277-458fee82e534</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Hall, Kyle</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>6a6908af-8856-431e-8277-458fee82e534</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: VanMaanen, Derek</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>6a6908af-8856-431e-8277-458fee82e534</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Whalen, Matthew</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>6a6908af-8856-431e-8277-458fee82e534</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Millard-Martin, Ben</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>324c5ae3-b0ac-4302-b701-598ebbb25870</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Oliver, Allison</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Contact missing affiliation: Frazer, Gordon W.</t>
         </is>
       </c>
     </row>

</xml_diff>